<commit_message>
Update FrName + FrCompositionDocument (#49) edf2bfc313cab10a92886f68b2170a0a9c4927ac
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-fr-bundle-document.xlsx
+++ b/main/ig/StructureDefinition-fr-bundle-document.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-08-25T15:42:10+00:00</t>
+    <t>2025-10-02T14:05:03+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -364,7 +364,7 @@
     <t>A human language.</t>
   </si>
   <si>
-    <t>http://hl7.org/fhir/ValueSet/languages</t>
+    <t>http://hl7.org/fhir/ValueSet/languages|4.0.1</t>
   </si>
   <si>
     <t>Resource.language</t>
@@ -4659,7 +4659,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="22" hidden="true">
+    <row r="22">
       <c r="A22" t="s" s="2">
         <v>189</v>
       </c>
@@ -8283,7 +8283,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="54" hidden="true">
+    <row r="54">
       <c r="A54" t="s" s="2">
         <v>275</v>
       </c>
@@ -11909,7 +11909,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="86" hidden="true">
+    <row r="86">
       <c r="A86" t="s" s="2">
         <v>314</v>
       </c>
@@ -15533,7 +15533,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="118" hidden="true">
+    <row r="118">
       <c r="A118" t="s" s="2">
         <v>353</v>
       </c>
@@ -19157,7 +19157,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="150" hidden="true">
+    <row r="150">
       <c r="A150" t="s" s="2">
         <v>391</v>
       </c>
@@ -22781,7 +22781,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="182" hidden="true">
+    <row r="182">
       <c r="A182" t="s" s="2">
         <v>427</v>
       </c>
@@ -26405,7 +26405,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="214" hidden="true">
+    <row r="214">
       <c r="A214" t="s" s="2">
         <v>465</v>
       </c>
@@ -30029,7 +30029,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="246" hidden="true">
+    <row r="246">
       <c r="A246" t="s" s="2">
         <v>502</v>
       </c>
@@ -33653,7 +33653,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="278" hidden="true">
+    <row r="278">
       <c r="A278" t="s" s="2">
         <v>540</v>
       </c>
@@ -37277,7 +37277,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="310" hidden="true">
+    <row r="310">
       <c r="A310" t="s" s="2">
         <v>577</v>
       </c>
@@ -40451,12 +40451,12 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:AN337">
-    <filterColumn colId="6">
+    <filterColumn colId="7">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
       </customFilters>
     </filterColumn>
-    <filterColumn colId="26">
+    <filterColumn colId="27">
       <filters blank="true"/>
     </filterColumn>
   </autoFilter>

</xml_diff>

<commit_message>
update FrDocumentDevice (#56) 0e5d0b73d7b8281f70eebda7c49450b3d0f88fa8
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-fr-bundle-document.xlsx
+++ b/main/ig/StructureDefinition-fr-bundle-document.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-10-02T14:05:03+00:00</t>
+    <t>2025-10-02T15:16:38+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1464,7 +1464,7 @@
     <t>Bundle.entry:device.resource</t>
   </si>
   <si>
-    <t xml:space="preserve">Device {https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-device-document}
+    <t xml:space="preserve">Device {https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-device-auteur-document}
 </t>
   </si>
   <si>

</xml_diff>

<commit_message>
Renommage entete fhir (#68)
* Renommage entete FHIR

* Renommage entete FHIR 38f2afd9a56603ba9de34ae56c3c5dee9efe2b94
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-fr-bundle-document.xlsx
+++ b/main/ig/StructureDefinition-fr-bundle-document.xlsx
@@ -39,13 +39,13 @@
     <t>Name</t>
   </si>
   <si>
-    <t>FrBundleDocument</t>
+    <t>FRBundleDocument</t>
   </si>
   <si>
     <t>Title</t>
   </si>
   <si>
-    <t>Fr Bundle Document</t>
+    <t>FR Bundle Document</t>
   </si>
   <si>
     <t>Status</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-10-21T17:18:21+00:00</t>
+    <t>2025-10-22T08:56:46+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -576,7 +576,7 @@
     <t>7</t>
   </si>
   <si>
-    <t>Ressource Entry dans le FrBundleDocument</t>
+    <t>Ressource Entry dans le FRBundleDocument</t>
   </si>
   <si>
     <t>Une ressource Entry incluse dans le bundle de ressources du document</t>

</xml_diff>